<commit_message>
Footer: stop the leading-dot fix from oscillating; record staging and production results
On a 412 px phone one footer line on gokesari.com began with "·". Hiding a
line's leading dot let that link fit on the line above, where it needed its
dot back, so a single measuring pass left either a stray dot or a missing
one. Lines are now measured with every dot shown and pinned with a
zero-height break, so dropping the leading dot only shortens its line.
Re-measures on width change and when the web font arrives.

New E2E check sweeps 320-1366 px; it fails on the live footer and passes
with the fix (18/18 on a local production build).

Test results and the status report now carry the staging re-check after
#147/#148 and the production release and smoke test (PR #149).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014VPELLzkzgr6rEhrzWyDHd
</commit_message>
<xml_diff>
--- a/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-13.xlsx
+++ b/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-13.xlsx
@@ -503,7 +503,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Not run</t>
+          <t>Not run (code shipped inert, DB_SPLIT_MODE=single)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -535,17 +535,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Deployed; page OK; photo read hit 504 on Hostinger</t>
+          <t>PASS after #147/#148: upload 201 in 31 s, type-the-details, CONFIRMED; OCR worker does not start on Hostinger</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Not released</t>
+          <t>LIVE 13 Oct (PR #149); routes answer 307/401 when signed out</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>PR #147 (25 s limit + type-the-details fallback + health check) → re-test</t>
+          <t>Open: OCR worker start on Hostinger (owners type details meanwhile)</t>
         </is>
       </c>
     </row>
@@ -577,7 +577,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Not released</t>
+          <t>LIVE 13 Oct (rule on)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -614,12 +614,12 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Not released</t>
+          <t>LIVE 13 Oct; E2E 16/16 on gokesari.com</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Stray "·" on one phone line found on production → follow-up PR (fix + width-sweep test)</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Not released</t>
+          <t>LIVE 13 Oct; E2E 16/16 on gokesari.com</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Reaches apps with the site (no store release)</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -720,12 +720,12 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Branding E2E only so far</t>
+          <t>Branding E2E 16/16; upload flow; CI green on release</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Smoke: 8 public pages 200 before and after; branding E2E 16/16</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">

</xml_diff>